<commit_message>
Sync database backups and processed timestamps
</commit_message>
<xml_diff>
--- a/Newdata/已撥缺料.XLSX
+++ b/Newdata/已撥缺料.XLSX
@@ -11,351 +11,429 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="765" uniqueCount="140">
-  <si>
-    <t>200006299</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1005" uniqueCount="166">
+  <si>
+    <t>200006366</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>080100152306</t>
+    <t>4023000061C0</t>
+  </si>
+  <si>
+    <t>0060</t>
+  </si>
+  <si>
+    <t>EA</t>
+  </si>
+  <si>
+    <t>油壓缸/打刀油缸_行程14</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>0010</t>
+  </si>
+  <si>
+    <t>SHEO</t>
+  </si>
+  <si>
+    <t>0101</t>
+  </si>
+  <si>
+    <t>1F004</t>
+  </si>
+  <si>
+    <t>組件課</t>
+  </si>
+  <si>
+    <t>REL</t>
+  </si>
+  <si>
+    <t>9804</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>8429000727A0</t>
+  </si>
+  <si>
+    <t>0080</t>
+  </si>
+  <si>
+    <t>彈簧座_d22*D32*16</t>
+  </si>
+  <si>
+    <t>0100</t>
+  </si>
+  <si>
+    <t>200006367</t>
+  </si>
+  <si>
+    <t>8423000097A2</t>
+  </si>
+  <si>
+    <t>0420</t>
+  </si>
+  <si>
+    <t>吹氣環_d127xD138x14H</t>
+  </si>
+  <si>
+    <t>0102</t>
+  </si>
+  <si>
+    <t>3154001543B3</t>
+  </si>
+  <si>
+    <t>0440</t>
+  </si>
+  <si>
+    <t>主軸前蓋_d127*D195*33L</t>
+  </si>
+  <si>
+    <t>200006368</t>
+  </si>
+  <si>
+    <t>080100113204</t>
+  </si>
+  <si>
+    <t>G6K 主軸,021305_BT50,CW45</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>0802</t>
+  </si>
+  <si>
+    <t>200006370</t>
+  </si>
+  <si>
+    <t>080100033903</t>
+  </si>
+  <si>
+    <t>G2.5K主軸,010830_BT50,C0DIN</t>
+  </si>
+  <si>
+    <t>1X001</t>
+  </si>
+  <si>
+    <t>虛擬工作中心</t>
+  </si>
+  <si>
+    <t>200006371</t>
+  </si>
+  <si>
+    <t>3154001366C1</t>
+  </si>
+  <si>
+    <t>0290</t>
+  </si>
+  <si>
+    <t>主軸前蓋_246*430*79</t>
+  </si>
+  <si>
+    <t>200006385</t>
+  </si>
+  <si>
+    <t>8310000702A1</t>
+  </si>
+  <si>
+    <t>0170</t>
+  </si>
+  <si>
+    <t>馬達座_G8K-a22</t>
+  </si>
+  <si>
+    <t>0104</t>
+  </si>
+  <si>
+    <t>200006390</t>
+  </si>
+  <si>
+    <t>4023000108B0</t>
+  </si>
+  <si>
+    <t>0370</t>
+  </si>
+  <si>
+    <t>打刀油缸_83-62-12</t>
+  </si>
+  <si>
+    <t>200006423</t>
+  </si>
+  <si>
+    <t>0360</t>
+  </si>
+  <si>
+    <t>0380</t>
+  </si>
+  <si>
+    <t>200006431</t>
+  </si>
+  <si>
+    <t>200006432</t>
+  </si>
+  <si>
+    <t>080100120402</t>
+  </si>
+  <si>
+    <t>0050</t>
+  </si>
+  <si>
+    <t>G8K 主軸,021387_BT50,0W45</t>
+  </si>
+  <si>
+    <t>200006433</t>
+  </si>
+  <si>
+    <t>200006452</t>
+  </si>
+  <si>
+    <t>080100023404</t>
+  </si>
+  <si>
+    <t>0040</t>
+  </si>
+  <si>
+    <t>G6K 主軸,021327_BT50,C0DIN</t>
+  </si>
+  <si>
+    <t>200006454</t>
+  </si>
+  <si>
+    <t>8814001415C0</t>
+  </si>
+  <si>
+    <t>0240</t>
+  </si>
+  <si>
+    <t>機頭加工圖,#50G6K_HCMC-1100</t>
+  </si>
+  <si>
+    <t>06</t>
+  </si>
+  <si>
+    <t>200006456</t>
+  </si>
+  <si>
+    <t>8814001018A1</t>
+  </si>
+  <si>
+    <t>0270</t>
+  </si>
+  <si>
+    <t>機頭滑座加工圖_PI-1,Z780</t>
+  </si>
+  <si>
+    <t>200006460</t>
+  </si>
+  <si>
+    <t>200006466</t>
+  </si>
+  <si>
+    <t>8916000299A1</t>
+  </si>
+  <si>
+    <t>0450</t>
+  </si>
+  <si>
+    <t>防濺護罩,左/AHC用_d532*108H</t>
+  </si>
+  <si>
+    <t>0107</t>
+  </si>
+  <si>
+    <t>9816</t>
+  </si>
+  <si>
+    <t>200006471</t>
+  </si>
+  <si>
+    <t>8342000234A0</t>
+  </si>
+  <si>
+    <t>0190</t>
+  </si>
+  <si>
+    <t>吊桿螺帽_M16*25*8</t>
+  </si>
+  <si>
+    <t>3214000289B0</t>
+  </si>
+  <si>
+    <t>0210</t>
+  </si>
+  <si>
+    <t>吊桿,DDS20K_MVP-8</t>
+  </si>
+  <si>
+    <t>3154001577B0</t>
+  </si>
+  <si>
+    <t>0430</t>
+  </si>
+  <si>
+    <t>主軸前蓋_d82.5*D148*H28</t>
+  </si>
+  <si>
+    <t>200006475</t>
+  </si>
+  <si>
+    <t>080100050201</t>
+  </si>
+  <si>
+    <t>0030</t>
+  </si>
+  <si>
+    <t>D20K 主軸,010683_A63,M50,C0</t>
+  </si>
+  <si>
+    <t>8310000667A1</t>
+  </si>
+  <si>
+    <t>馬達固定座_HSA2215/20KRPM</t>
+  </si>
+  <si>
+    <t>200006476</t>
+  </si>
+  <si>
+    <t>8420002210A0</t>
+  </si>
+  <si>
+    <t>0230</t>
+  </si>
+  <si>
+    <t>下間隔環組,DDS20K_d65*D100*18</t>
+  </si>
+  <si>
+    <t>5063000121B0</t>
+  </si>
+  <si>
+    <t>0310</t>
+  </si>
+  <si>
+    <t>油壓缸活塞,DDS20K_MVP-8(D100*d70*63.5H)</t>
+  </si>
+  <si>
+    <t>200006486</t>
+  </si>
+  <si>
+    <t>200006487</t>
+  </si>
+  <si>
+    <t>200006488</t>
+  </si>
+  <si>
+    <t>3241000017A1</t>
+  </si>
+  <si>
+    <t>直齒離合器,C軸2.5度_D330*d280*H40,144T</t>
+  </si>
+  <si>
+    <t>8319000682A0</t>
+  </si>
+  <si>
+    <t>金屬墊片,A軸軸承箱用_d142*D186*4t</t>
+  </si>
+  <si>
+    <t>892300066700</t>
+  </si>
+  <si>
+    <t>0610</t>
+  </si>
+  <si>
+    <t>出貨固定板_EA/EAY,HF-AU</t>
+  </si>
+  <si>
+    <t>200006495</t>
+  </si>
+  <si>
+    <t>200006496</t>
+  </si>
+  <si>
+    <t>305000001101</t>
+  </si>
+  <si>
+    <t>陶珠軸承_FAG-HC7014C.T.P4S.UL,2個1組</t>
+  </si>
+  <si>
+    <t>EC210689</t>
+  </si>
+  <si>
+    <t>0128</t>
+  </si>
+  <si>
+    <t>305000001201</t>
   </si>
   <si>
     <t>0020</t>
   </si>
   <si>
-    <t>EA</t>
-  </si>
-  <si>
-    <t>DA15K 主軸,021856_BT40,M60,CWDIN</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>0010</t>
-  </si>
-  <si>
-    <t>SHEO</t>
-  </si>
-  <si>
-    <t>50</t>
-  </si>
-  <si>
-    <t>1F004</t>
-  </si>
-  <si>
-    <t>組件課</t>
-  </si>
-  <si>
-    <t>REL</t>
-  </si>
-  <si>
-    <t>0802</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>200006330</t>
-  </si>
-  <si>
-    <t>080100036004</t>
-  </si>
-  <si>
-    <t>0040</t>
-  </si>
-  <si>
-    <t>G6K 主軸,021327_BBT50,C045</t>
-  </si>
-  <si>
-    <t>200006367</t>
-  </si>
-  <si>
-    <t>303500039801</t>
-  </si>
-  <si>
-    <t>單列斜角滾珠軸承_FAG-HS7018C.T.P4S.UL,2個1組</t>
-  </si>
-  <si>
-    <t>0128</t>
-  </si>
-  <si>
-    <t>9804</t>
-  </si>
-  <si>
-    <t>8420002329A1</t>
-  </si>
-  <si>
-    <t>0290</t>
-  </si>
-  <si>
-    <t>間隔環,前內_d90.5*D113*24,HSA2215</t>
-  </si>
-  <si>
-    <t>0102</t>
-  </si>
-  <si>
-    <t>8420002330A1</t>
-  </si>
-  <si>
-    <t>0300</t>
-  </si>
-  <si>
-    <t>間隔環,前外_d117*D140*24,HSA2215</t>
-  </si>
-  <si>
-    <t>8423000097A2</t>
-  </si>
-  <si>
-    <t>0420</t>
-  </si>
-  <si>
-    <t>吹氣環_d127xD138x14H</t>
-  </si>
-  <si>
-    <t>3154001543B3</t>
-  </si>
-  <si>
-    <t>0440</t>
-  </si>
-  <si>
-    <t>主軸前蓋_d127*D195*33L</t>
-  </si>
-  <si>
-    <t>200006368</t>
-  </si>
-  <si>
-    <t>080100113204</t>
-  </si>
-  <si>
-    <t>0060</t>
-  </si>
-  <si>
-    <t>G6K 主軸,021305_BT50,CW45</t>
-  </si>
-  <si>
-    <t>8814001257B3</t>
-  </si>
-  <si>
-    <t>0170</t>
-  </si>
-  <si>
-    <t>機頭加工圖,G6K_HCMC-2110</t>
-  </si>
-  <si>
-    <t>06</t>
-  </si>
-  <si>
-    <t>200006370</t>
-  </si>
-  <si>
-    <t>080100033903</t>
-  </si>
-  <si>
-    <t>0080</t>
-  </si>
-  <si>
-    <t>G2.5K主軸,010830_BT50,C0DIN</t>
-  </si>
-  <si>
-    <t>1X001</t>
-  </si>
-  <si>
-    <t>虛擬工作中心</t>
-  </si>
-  <si>
-    <t>8921000777A0</t>
-  </si>
-  <si>
-    <t>0110</t>
-  </si>
-  <si>
-    <t>感應器支撐架_D30104H,D70*10H</t>
-  </si>
-  <si>
-    <t>0101</t>
-  </si>
-  <si>
-    <t>8016001298A0</t>
-  </si>
-  <si>
-    <t>0260</t>
-  </si>
-  <si>
-    <t>板金架_L765xW152xH38</t>
-  </si>
-  <si>
-    <t>0107</t>
-  </si>
-  <si>
-    <t>9801</t>
-  </si>
-  <si>
-    <t>200006371</t>
-  </si>
-  <si>
-    <t>3154001366C1</t>
-  </si>
-  <si>
-    <t>主軸前蓋_246*430*79</t>
-  </si>
-  <si>
-    <t>200006375</t>
-  </si>
-  <si>
-    <t>8420002327A0</t>
-  </si>
-  <si>
-    <t>0330</t>
-  </si>
-  <si>
-    <t>間隔環,前下_d90*D129*13.5,HSA2215</t>
-  </si>
-  <si>
-    <t>0350</t>
-  </si>
-  <si>
-    <t>0360</t>
-  </si>
-  <si>
-    <t>200006377</t>
-  </si>
-  <si>
-    <t>305000001101</t>
-  </si>
-  <si>
-    <t>陶珠軸承_FAG-HC7014C.T.P4S.UL,2個1組</t>
-  </si>
-  <si>
-    <t>EC210689</t>
-  </si>
-  <si>
-    <t>321400027300</t>
-  </si>
-  <si>
-    <t>抓刀筒夾,OTT_BT40</t>
+    <t>陶珠軸承_FAG-HC7013C.T.P4S.UL,2個1組</t>
+  </si>
+  <si>
+    <t>111400007900</t>
+  </si>
+  <si>
+    <t>0180</t>
+  </si>
+  <si>
+    <t>盤型彈簧/左旋_40-20-1</t>
   </si>
   <si>
     <t>0120</t>
   </si>
   <si>
-    <t>0801</t>
-  </si>
-  <si>
-    <t>305000001201</t>
-  </si>
-  <si>
-    <t>陶珠軸承_FAG-HC7013C.T.P4S.UL,2個1組</t>
-  </si>
-  <si>
-    <t>200006385</t>
-  </si>
-  <si>
-    <t>080100022704</t>
-  </si>
-  <si>
-    <t>0050</t>
-  </si>
-  <si>
-    <t>G6K 主軸,021327_BT50,0045</t>
-  </si>
-  <si>
-    <t>8310000702A1</t>
-  </si>
-  <si>
-    <t>馬達座_G8K-a22</t>
-  </si>
-  <si>
-    <t>0104</t>
-  </si>
-  <si>
-    <t>200006404</t>
-  </si>
-  <si>
-    <t>200006423</t>
-  </si>
-  <si>
-    <t>0380</t>
-  </si>
-  <si>
-    <t>200006431</t>
-  </si>
-  <si>
-    <t>200006432</t>
-  </si>
-  <si>
-    <t>080100120402</t>
-  </si>
-  <si>
-    <t>G8K 主軸,021387_BT50,0W45</t>
-  </si>
-  <si>
-    <t>200006433</t>
-  </si>
-  <si>
-    <t>200006454</t>
-  </si>
-  <si>
-    <t>8814001415C0</t>
-  </si>
-  <si>
-    <t>0240</t>
-  </si>
-  <si>
-    <t>機頭加工圖,#50G6K_HCMC-1100</t>
-  </si>
-  <si>
-    <t>200006470</t>
-  </si>
-  <si>
-    <t>3227000055C0</t>
-  </si>
-  <si>
-    <t>0100</t>
-  </si>
-  <si>
-    <t>撓性聯軸器,ROTEX_98ShA-GS6.0-d38,6.0P-d50</t>
-  </si>
-  <si>
-    <t>200006475</t>
-  </si>
-  <si>
-    <t>080100050201</t>
-  </si>
-  <si>
-    <t>0030</t>
-  </si>
-  <si>
-    <t>D20K 主軸,010683_A63,M50,C0</t>
-  </si>
-  <si>
-    <t>8311000415A0</t>
-  </si>
-  <si>
-    <t>前油箱蓋板_195*160*15</t>
-  </si>
-  <si>
-    <t>8310000667A1</t>
-  </si>
-  <si>
-    <t>馬達固定座_HSA2215/20KRPM</t>
-  </si>
-  <si>
-    <t>8814001399A4</t>
-  </si>
-  <si>
-    <t>機頭加工圖,Z780_#40,D20K</t>
-  </si>
-  <si>
-    <t>630000329</t>
-  </si>
-  <si>
-    <t>2050000123A2</t>
-  </si>
-  <si>
-    <t>中間軸齒輪_m2.5*72t*25w</t>
+    <t>200006502</t>
+  </si>
+  <si>
+    <t>305000004501</t>
+  </si>
+  <si>
+    <t>陶珠軸承_FAG-HC7013E.T.P4S.UL,2個1組</t>
+  </si>
+  <si>
+    <t>0200</t>
+  </si>
+  <si>
+    <t>5063000120A0</t>
+  </si>
+  <si>
+    <t>0220</t>
+  </si>
+  <si>
+    <t>油壓缸外蓋,DDS20K_MVP-8(D100*d70*H64)</t>
+  </si>
+  <si>
+    <t>5063000163B0</t>
+  </si>
+  <si>
+    <t>油壓缸底蓋_MVP-10</t>
+  </si>
+  <si>
+    <t>630000333</t>
+  </si>
+  <si>
+    <t>080200555000</t>
+  </si>
+  <si>
+    <t>0070</t>
+  </si>
+  <si>
+    <t>MVP-8機頭D15K,021581_#40,38F18,C,AT8</t>
+  </si>
+  <si>
+    <t>630000338</t>
+  </si>
+  <si>
+    <t>080100084704</t>
+  </si>
+  <si>
+    <t>D15K 主軸,010017_BT40,M60,CWDIN</t>
   </si>
   <si>
     <t>訂單</t>
@@ -535,7 +613,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:Y38"/>
+  <dimension ref="A1:Y50"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="11" customWidth="1"/>
@@ -547,7 +625,7 @@
     <col min="7" max="7" bestFit="1" width="10" customWidth="1"/>
     <col min="8" max="8" bestFit="1" width="10" customWidth="1"/>
     <col min="9" max="9" bestFit="1" width="12" customWidth="1"/>
-    <col min="10" max="10" bestFit="1" width="38" customWidth="1"/>
+    <col min="10" max="10" bestFit="1" width="36" customWidth="1"/>
     <col min="11" max="11" bestFit="1" width="4" customWidth="1"/>
     <col min="12" max="12" bestFit="1" width="6" customWidth="1"/>
     <col min="13" max="13" bestFit="1" width="6" customWidth="1"/>
@@ -567,79 +645,79 @@
   <sheetData>
     <row r="1" spans="1:25">
       <c r="A1" s="1" t="s">
-        <v>115</v>
+        <v>141</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>116</v>
+        <v>142</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>117</v>
+        <v>143</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>118</v>
+        <v>144</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>119</v>
+        <v>145</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>120</v>
+        <v>146</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>121</v>
+        <v>147</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>122</v>
+        <v>148</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>123</v>
+        <v>149</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>125</v>
+        <v>151</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>126</v>
+        <v>152</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>128</v>
+        <v>154</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>129</v>
+        <v>155</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>130</v>
+        <v>156</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>131</v>
+        <v>157</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>132</v>
+        <v>158</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>133</v>
+        <v>159</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>134</v>
+        <v>160</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>135</v>
+        <v>161</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>136</v>
+        <v>162</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>137</v>
+        <v>163</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>138</v>
+        <v>164</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>139</v>
+        <v>165</v>
       </c>
     </row>
     <row r="2" spans="1:25">
@@ -656,7 +734,7 @@
         <v>3</v>
       </c>
       <c r="E2" s="2">
-        <v>46059</v>
+        <v>46091</v>
       </c>
       <c r="F2" s="3">
         <v>1</v>
@@ -721,49 +799,49 @@
     </row>
     <row r="3" spans="1:25">
       <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
         <v>15</v>
       </c>
-      <c r="B3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>16</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" s="2">
+        <v>46091</v>
+      </c>
+      <c r="F3" s="3">
+        <v>2</v>
+      </c>
+      <c r="G3" s="3">
+        <v>0</v>
+      </c>
+      <c r="H3" s="3">
+        <v>2</v>
+      </c>
+      <c r="I3" t="s">
+        <v>4</v>
+      </c>
+      <c r="J3" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="2">
-        <v>46034</v>
-      </c>
-      <c r="F3" s="3">
-        <v>1</v>
-      </c>
-      <c r="G3" s="3">
-        <v>0</v>
-      </c>
-      <c r="H3" s="3">
-        <v>1</v>
-      </c>
-      <c r="I3" t="s">
-        <v>4</v>
-      </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
+        <v>6</v>
+      </c>
+      <c r="L3" t="s">
+        <v>7</v>
+      </c>
+      <c r="M3" t="s">
+        <v>8</v>
+      </c>
+      <c r="N3" t="s">
+        <v>1</v>
+      </c>
+      <c r="O3" t="s">
         <v>18</v>
-      </c>
-      <c r="K3" t="s">
-        <v>6</v>
-      </c>
-      <c r="L3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M3" t="s">
-        <v>8</v>
-      </c>
-      <c r="N3" t="s">
-        <v>1</v>
-      </c>
-      <c r="O3" t="s">
-        <v>9</v>
       </c>
       <c r="P3" t="s">
         <v>10</v>
@@ -775,7 +853,7 @@
         <v>1</v>
       </c>
       <c r="S3" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T3" t="s">
         <v>12</v>
@@ -807,25 +885,25 @@
         <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E4" s="2">
         <v>46086</v>
       </c>
       <c r="F4" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G4" s="3">
         <v>0</v>
       </c>
       <c r="H4" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I4" t="s">
         <v>4</v>
       </c>
       <c r="J4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K4" t="s">
         <v>6</v>
@@ -840,7 +918,7 @@
         <v>1</v>
       </c>
       <c r="O4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P4" t="s">
         <v>10</v>
@@ -852,13 +930,13 @@
         <v>1</v>
       </c>
       <c r="S4" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T4" t="s">
         <v>12</v>
       </c>
       <c r="U4" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="V4" t="s">
         <v>1</v>
@@ -917,7 +995,7 @@
         <v>1</v>
       </c>
       <c r="O5" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="P5" t="s">
         <v>10</v>
@@ -935,7 +1013,7 @@
         <v>12</v>
       </c>
       <c r="U5" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="V5" t="s">
         <v>1</v>
@@ -952,7 +1030,7 @@
     </row>
     <row r="6" spans="1:25">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s">
         <v>1</v>
@@ -961,40 +1039,40 @@
         <v>28</v>
       </c>
       <c r="D6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" s="2">
+        <v>46101</v>
+      </c>
+      <c r="F6" s="3">
+        <v>1</v>
+      </c>
+      <c r="G6" s="3">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3">
+        <v>1</v>
+      </c>
+      <c r="I6" t="s">
+        <v>4</v>
+      </c>
+      <c r="J6" t="s">
         <v>29</v>
       </c>
-      <c r="E6" s="2">
-        <v>46086</v>
-      </c>
-      <c r="F6" s="3">
-        <v>1</v>
-      </c>
-      <c r="G6" s="3">
-        <v>0</v>
-      </c>
-      <c r="H6" s="3">
-        <v>1</v>
-      </c>
-      <c r="I6" t="s">
-        <v>4</v>
-      </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
+        <v>6</v>
+      </c>
+      <c r="L6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M6" t="s">
+        <v>8</v>
+      </c>
+      <c r="N6" t="s">
+        <v>1</v>
+      </c>
+      <c r="O6" t="s">
         <v>30</v>
-      </c>
-      <c r="K6" t="s">
-        <v>6</v>
-      </c>
-      <c r="L6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M6" t="s">
-        <v>8</v>
-      </c>
-      <c r="N6" t="s">
-        <v>1</v>
-      </c>
-      <c r="O6" t="s">
-        <v>27</v>
       </c>
       <c r="P6" t="s">
         <v>10</v>
@@ -1012,7 +1090,7 @@
         <v>12</v>
       </c>
       <c r="U6" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="V6" t="s">
         <v>1</v>
@@ -1029,67 +1107,67 @@
     </row>
     <row r="7" spans="1:25">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="B7" t="s">
         <v>1</v>
       </c>
       <c r="C7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="2">
+        <v>46064</v>
+      </c>
+      <c r="F7" s="3">
+        <v>1</v>
+      </c>
+      <c r="G7" s="3">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3">
+        <v>1</v>
+      </c>
+      <c r="I7" t="s">
+        <v>4</v>
+      </c>
+      <c r="J7" t="s">
+        <v>34</v>
+      </c>
+      <c r="K7" t="s">
+        <v>6</v>
+      </c>
+      <c r="L7" t="s">
+        <v>7</v>
+      </c>
+      <c r="M7" t="s">
+        <v>8</v>
+      </c>
+      <c r="N7" t="s">
+        <v>1</v>
+      </c>
+      <c r="O7" t="s">
+        <v>30</v>
+      </c>
+      <c r="P7" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>36</v>
+      </c>
+      <c r="R7" t="s">
+        <v>1</v>
+      </c>
+      <c r="S7" s="3">
+        <v>1</v>
+      </c>
+      <c r="T7" t="s">
+        <v>12</v>
+      </c>
+      <c r="U7" t="s">
         <v>31</v>
-      </c>
-      <c r="D7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E7" s="2">
-        <v>46086</v>
-      </c>
-      <c r="F7" s="3">
-        <v>1</v>
-      </c>
-      <c r="G7" s="3">
-        <v>0</v>
-      </c>
-      <c r="H7" s="3">
-        <v>1</v>
-      </c>
-      <c r="I7" t="s">
-        <v>4</v>
-      </c>
-      <c r="J7" t="s">
-        <v>33</v>
-      </c>
-      <c r="K7" t="s">
-        <v>6</v>
-      </c>
-      <c r="L7" t="s">
-        <v>7</v>
-      </c>
-      <c r="M7" t="s">
-        <v>8</v>
-      </c>
-      <c r="N7" t="s">
-        <v>1</v>
-      </c>
-      <c r="O7" t="s">
-        <v>27</v>
-      </c>
-      <c r="P7" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>11</v>
-      </c>
-      <c r="R7" t="s">
-        <v>1</v>
-      </c>
-      <c r="S7" s="3">
-        <v>1</v>
-      </c>
-      <c r="T7" t="s">
-        <v>12</v>
-      </c>
-      <c r="U7" t="s">
-        <v>23</v>
       </c>
       <c r="V7" t="s">
         <v>1</v>
@@ -1106,19 +1184,19 @@
     </row>
     <row r="8" spans="1:25">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="B8" t="s">
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E8" s="2">
-        <v>46086</v>
+        <v>46052</v>
       </c>
       <c r="F8" s="3">
         <v>1</v>
@@ -1133,7 +1211,7 @@
         <v>4</v>
       </c>
       <c r="J8" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="K8" t="s">
         <v>6</v>
@@ -1148,7 +1226,7 @@
         <v>1</v>
       </c>
       <c r="O8" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="P8" t="s">
         <v>10</v>
@@ -1166,7 +1244,7 @@
         <v>12</v>
       </c>
       <c r="U8" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="V8" t="s">
         <v>1</v>
@@ -1183,19 +1261,19 @@
     </row>
     <row r="9" spans="1:25">
       <c r="A9" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B9" t="s">
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D9" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E9" s="2">
-        <v>46101</v>
+        <v>46063</v>
       </c>
       <c r="F9" s="3">
         <v>1</v>
@@ -1210,7 +1288,7 @@
         <v>4</v>
       </c>
       <c r="J9" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="K9" t="s">
         <v>6</v>
@@ -1225,7 +1303,7 @@
         <v>1</v>
       </c>
       <c r="O9" t="s">
-        <v>9</v>
+        <v>45</v>
       </c>
       <c r="P9" t="s">
         <v>10</v>
@@ -1260,19 +1338,19 @@
     </row>
     <row r="10" spans="1:25">
       <c r="A10" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="B10" t="s">
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="D10" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E10" s="2">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="F10" s="3">
         <v>1</v>
@@ -1287,7 +1365,7 @@
         <v>4</v>
       </c>
       <c r="J10" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="K10" t="s">
         <v>6</v>
@@ -1302,7 +1380,7 @@
         <v>1</v>
       </c>
       <c r="O10" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="P10" t="s">
         <v>10</v>
@@ -1320,7 +1398,7 @@
         <v>12</v>
       </c>
       <c r="U10" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="V10" t="s">
         <v>1</v>
@@ -1337,19 +1415,19 @@
     </row>
     <row r="11" spans="1:25">
       <c r="A11" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B11" t="s">
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E11" s="2">
-        <v>46064</v>
+        <v>46041</v>
       </c>
       <c r="F11" s="3">
         <v>1</v>
@@ -1364,7 +1442,7 @@
         <v>4</v>
       </c>
       <c r="J11" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="K11" t="s">
         <v>6</v>
@@ -1379,13 +1457,13 @@
         <v>1</v>
       </c>
       <c r="O11" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="P11" t="s">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="Q11" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="R11" t="s">
         <v>1</v>
@@ -1414,19 +1492,19 @@
     </row>
     <row r="12" spans="1:25">
       <c r="A12" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B12" t="s">
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="D12" t="s">
         <v>52</v>
       </c>
       <c r="E12" s="2">
-        <v>46064</v>
+        <v>46041</v>
       </c>
       <c r="F12" s="3">
         <v>1</v>
@@ -1441,7 +1519,7 @@
         <v>4</v>
       </c>
       <c r="J12" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="K12" t="s">
         <v>6</v>
@@ -1456,13 +1534,13 @@
         <v>1</v>
       </c>
       <c r="O12" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="P12" t="s">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="Q12" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="R12" t="s">
         <v>1</v>
@@ -1474,7 +1552,7 @@
         <v>12</v>
       </c>
       <c r="U12" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="V12" t="s">
         <v>1</v>
@@ -1491,19 +1569,19 @@
     </row>
     <row r="13" spans="1:25">
       <c r="A13" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="B13" t="s">
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="D13" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E13" s="2">
-        <v>46064</v>
+        <v>46034</v>
       </c>
       <c r="F13" s="3">
         <v>1</v>
@@ -1518,7 +1596,7 @@
         <v>4</v>
       </c>
       <c r="J13" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="K13" t="s">
         <v>6</v>
@@ -1533,13 +1611,13 @@
         <v>1</v>
       </c>
       <c r="O13" t="s">
-        <v>58</v>
+        <v>23</v>
       </c>
       <c r="P13" t="s">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="Q13" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="R13" t="s">
         <v>1</v>
@@ -1551,7 +1629,7 @@
         <v>12</v>
       </c>
       <c r="U13" t="s">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="V13" t="s">
         <v>1</v>
@@ -1568,19 +1646,19 @@
     </row>
     <row r="14" spans="1:25">
       <c r="A14" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B14" t="s">
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="D14" t="s">
-        <v>25</v>
+        <v>56</v>
       </c>
       <c r="E14" s="2">
-        <v>46052</v>
+        <v>46078</v>
       </c>
       <c r="F14" s="3">
         <v>1</v>
@@ -1595,7 +1673,7 @@
         <v>4</v>
       </c>
       <c r="J14" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="K14" t="s">
         <v>6</v>
@@ -1610,7 +1688,7 @@
         <v>1</v>
       </c>
       <c r="O14" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="P14" t="s">
         <v>10</v>
@@ -1628,7 +1706,7 @@
         <v>12</v>
       </c>
       <c r="U14" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="V14" t="s">
         <v>1</v>
@@ -1645,19 +1723,19 @@
     </row>
     <row r="15" spans="1:25">
       <c r="A15" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="B15" t="s">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="D15" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="E15" s="2">
-        <v>46100</v>
+        <v>46063</v>
       </c>
       <c r="F15" s="3">
         <v>1</v>
@@ -1672,7 +1750,7 @@
         <v>4</v>
       </c>
       <c r="J15" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="K15" t="s">
         <v>6</v>
@@ -1687,7 +1765,7 @@
         <v>1</v>
       </c>
       <c r="O15" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="P15" t="s">
         <v>10</v>
@@ -1705,7 +1783,7 @@
         <v>12</v>
       </c>
       <c r="U15" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="V15" t="s">
         <v>1</v>
@@ -1722,7 +1800,7 @@
     </row>
     <row r="16" spans="1:25">
       <c r="A16" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="B16" t="s">
         <v>1</v>
@@ -1731,10 +1809,10 @@
         <v>24</v>
       </c>
       <c r="D16" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="E16" s="2">
-        <v>46100</v>
+        <v>46063</v>
       </c>
       <c r="F16" s="3">
         <v>1</v>
@@ -1764,7 +1842,7 @@
         <v>1</v>
       </c>
       <c r="O16" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="P16" t="s">
         <v>10</v>
@@ -1782,7 +1860,7 @@
         <v>12</v>
       </c>
       <c r="U16" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="V16" t="s">
         <v>1</v>
@@ -1799,19 +1877,19 @@
     </row>
     <row r="17" spans="1:25">
       <c r="A17" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B17" t="s">
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>28</v>
+        <v>60</v>
       </c>
       <c r="D17" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="E17" s="2">
-        <v>46100</v>
+        <v>46079</v>
       </c>
       <c r="F17" s="3">
         <v>1</v>
@@ -1826,22 +1904,22 @@
         <v>4</v>
       </c>
       <c r="J17" t="s">
+        <v>62</v>
+      </c>
+      <c r="K17" t="s">
+        <v>6</v>
+      </c>
+      <c r="L17" t="s">
+        <v>7</v>
+      </c>
+      <c r="M17" t="s">
+        <v>8</v>
+      </c>
+      <c r="N17" t="s">
+        <v>1</v>
+      </c>
+      <c r="O17" t="s">
         <v>30</v>
-      </c>
-      <c r="K17" t="s">
-        <v>6</v>
-      </c>
-      <c r="L17" t="s">
-        <v>7</v>
-      </c>
-      <c r="M17" t="s">
-        <v>8</v>
-      </c>
-      <c r="N17" t="s">
-        <v>1</v>
-      </c>
-      <c r="O17" t="s">
-        <v>27</v>
       </c>
       <c r="P17" t="s">
         <v>10</v>
@@ -1859,7 +1937,7 @@
         <v>12</v>
       </c>
       <c r="U17" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="V17" t="s">
         <v>1</v>
@@ -1876,19 +1954,19 @@
     </row>
     <row r="18" spans="1:25">
       <c r="A18" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="B18" t="s">
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="D18" t="s">
-        <v>7</v>
+        <v>65</v>
       </c>
       <c r="E18" s="2">
-        <v>46048</v>
+        <v>46065</v>
       </c>
       <c r="F18" s="3">
         <v>1</v>
@@ -1903,7 +1981,7 @@
         <v>4</v>
       </c>
       <c r="J18" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="K18" t="s">
         <v>6</v>
@@ -1915,10 +1993,10 @@
         <v>8</v>
       </c>
       <c r="N18" t="s">
-        <v>72</v>
+        <v>1</v>
       </c>
       <c r="O18" t="s">
-        <v>22</v>
+        <v>67</v>
       </c>
       <c r="P18" t="s">
         <v>10</v>
@@ -1936,7 +2014,7 @@
         <v>12</v>
       </c>
       <c r="U18" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="V18" t="s">
         <v>1</v>
@@ -1953,19 +2031,19 @@
     </row>
     <row r="19" spans="1:25">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B19" t="s">
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="D19" t="s">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="E19" s="2">
-        <v>46048</v>
+        <v>46077</v>
       </c>
       <c r="F19" s="3">
         <v>1</v>
@@ -1980,7 +2058,7 @@
         <v>4</v>
       </c>
       <c r="J19" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="K19" t="s">
         <v>6</v>
@@ -1995,7 +2073,7 @@
         <v>1</v>
       </c>
       <c r="O19" t="s">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="P19" t="s">
         <v>10</v>
@@ -2007,13 +2085,13 @@
         <v>1</v>
       </c>
       <c r="S19" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T19" t="s">
         <v>12</v>
       </c>
       <c r="U19" t="s">
-        <v>76</v>
+        <v>31</v>
       </c>
       <c r="V19" t="s">
         <v>1</v>
@@ -2030,19 +2108,19 @@
     </row>
     <row r="20" spans="1:25">
       <c r="A20" t="s">
+        <v>68</v>
+      </c>
+      <c r="B20" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" t="s">
         <v>69</v>
       </c>
-      <c r="B20" t="s">
-        <v>1</v>
-      </c>
-      <c r="C20" t="s">
-        <v>77</v>
-      </c>
       <c r="D20" t="s">
-        <v>3</v>
+        <v>70</v>
       </c>
       <c r="E20" s="2">
-        <v>46048</v>
+        <v>46077</v>
       </c>
       <c r="F20" s="3">
         <v>1</v>
@@ -2057,7 +2135,7 @@
         <v>4</v>
       </c>
       <c r="J20" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="K20" t="s">
         <v>6</v>
@@ -2069,10 +2147,10 @@
         <v>8</v>
       </c>
       <c r="N20" t="s">
-        <v>72</v>
+        <v>1</v>
       </c>
       <c r="O20" t="s">
-        <v>22</v>
+        <v>67</v>
       </c>
       <c r="P20" t="s">
         <v>10</v>
@@ -2084,13 +2162,13 @@
         <v>1</v>
       </c>
       <c r="S20" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T20" t="s">
         <v>12</v>
       </c>
       <c r="U20" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="V20" t="s">
         <v>1</v>
@@ -2107,19 +2185,19 @@
     </row>
     <row r="21" spans="1:25">
       <c r="A21" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="B21" t="s">
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D21" t="s">
-        <v>81</v>
+        <v>3</v>
       </c>
       <c r="E21" s="2">
-        <v>46063</v>
+        <v>46085</v>
       </c>
       <c r="F21" s="3">
         <v>1</v>
@@ -2134,7 +2212,7 @@
         <v>4</v>
       </c>
       <c r="J21" t="s">
-        <v>82</v>
+        <v>5</v>
       </c>
       <c r="K21" t="s">
         <v>6</v>
@@ -2184,19 +2262,19 @@
     </row>
     <row r="22" spans="1:25">
       <c r="A22" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="B22" t="s">
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="D22" t="s">
-        <v>42</v>
+        <v>75</v>
       </c>
       <c r="E22" s="2">
-        <v>46063</v>
+        <v>46065</v>
       </c>
       <c r="F22" s="3">
         <v>1</v>
@@ -2211,7 +2289,7 @@
         <v>4</v>
       </c>
       <c r="J22" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="K22" t="s">
         <v>6</v>
@@ -2226,13 +2304,13 @@
         <v>1</v>
       </c>
       <c r="O22" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="P22" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="Q22" t="s">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="R22" t="s">
         <v>1</v>
@@ -2244,7 +2322,7 @@
         <v>12</v>
       </c>
       <c r="U22" t="s">
-        <v>23</v>
+        <v>78</v>
       </c>
       <c r="V22" t="s">
         <v>1</v>
@@ -2261,34 +2339,34 @@
     </row>
     <row r="23" spans="1:25">
       <c r="A23" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="B23" t="s">
         <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="D23" t="s">
-        <v>3</v>
+        <v>81</v>
       </c>
       <c r="E23" s="2">
-        <v>46038</v>
+        <v>46059</v>
       </c>
       <c r="F23" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G23" s="3">
         <v>0</v>
       </c>
       <c r="H23" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I23" t="s">
         <v>4</v>
       </c>
       <c r="J23" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="K23" t="s">
         <v>6</v>
@@ -2303,7 +2381,7 @@
         <v>1</v>
       </c>
       <c r="O23" t="s">
-        <v>75</v>
+        <v>23</v>
       </c>
       <c r="P23" t="s">
         <v>10</v>
@@ -2315,13 +2393,13 @@
         <v>1</v>
       </c>
       <c r="S23" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T23" t="s">
         <v>12</v>
       </c>
       <c r="U23" t="s">
-        <v>76</v>
+        <v>13</v>
       </c>
       <c r="V23" t="s">
         <v>1</v>
@@ -2338,19 +2416,19 @@
     </row>
     <row r="24" spans="1:25">
       <c r="A24" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="B24" t="s">
         <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>31</v>
+        <v>83</v>
       </c>
       <c r="D24" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="E24" s="2">
-        <v>46041</v>
+        <v>46059</v>
       </c>
       <c r="F24" s="3">
         <v>1</v>
@@ -2365,7 +2443,7 @@
         <v>4</v>
       </c>
       <c r="J24" t="s">
-        <v>33</v>
+        <v>85</v>
       </c>
       <c r="K24" t="s">
         <v>6</v>
@@ -2380,7 +2458,7 @@
         <v>1</v>
       </c>
       <c r="O24" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="P24" t="s">
         <v>10</v>
@@ -2398,7 +2476,7 @@
         <v>12</v>
       </c>
       <c r="U24" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="V24" t="s">
         <v>1</v>
@@ -2415,35 +2493,35 @@
     </row>
     <row r="25" spans="1:25">
       <c r="A25" t="s">
+        <v>79</v>
+      </c>
+      <c r="B25" t="s">
+        <v>1</v>
+      </c>
+      <c r="C25" t="s">
+        <v>86</v>
+      </c>
+      <c r="D25" t="s">
         <v>87</v>
       </c>
-      <c r="B25" t="s">
-        <v>1</v>
-      </c>
-      <c r="C25" t="s">
-        <v>34</v>
-      </c>
-      <c r="D25" t="s">
+      <c r="E25" s="2">
+        <v>46059</v>
+      </c>
+      <c r="F25" s="3">
+        <v>1</v>
+      </c>
+      <c r="G25" s="3">
+        <v>0</v>
+      </c>
+      <c r="H25" s="3">
+        <v>1</v>
+      </c>
+      <c r="I25" t="s">
+        <v>4</v>
+      </c>
+      <c r="J25" t="s">
         <v>88</v>
       </c>
-      <c r="E25" s="2">
-        <v>46041</v>
-      </c>
-      <c r="F25" s="3">
-        <v>1</v>
-      </c>
-      <c r="G25" s="3">
-        <v>0</v>
-      </c>
-      <c r="H25" s="3">
-        <v>1</v>
-      </c>
-      <c r="I25" t="s">
-        <v>4</v>
-      </c>
-      <c r="J25" t="s">
-        <v>36</v>
-      </c>
       <c r="K25" t="s">
         <v>6</v>
       </c>
@@ -2457,7 +2535,7 @@
         <v>1</v>
       </c>
       <c r="O25" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="P25" t="s">
         <v>10</v>
@@ -2475,7 +2553,7 @@
         <v>12</v>
       </c>
       <c r="U25" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="V25" t="s">
         <v>1</v>
@@ -2498,13 +2576,13 @@
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>34</v>
+        <v>90</v>
       </c>
       <c r="D26" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E26" s="2">
-        <v>46034</v>
+        <v>46050</v>
       </c>
       <c r="F26" s="3">
         <v>1</v>
@@ -2519,7 +2597,7 @@
         <v>4</v>
       </c>
       <c r="J26" t="s">
-        <v>36</v>
+        <v>92</v>
       </c>
       <c r="K26" t="s">
         <v>6</v>
@@ -2534,7 +2612,7 @@
         <v>1</v>
       </c>
       <c r="O26" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="P26" t="s">
         <v>10</v>
@@ -2546,13 +2624,13 @@
         <v>1</v>
       </c>
       <c r="S26" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T26" t="s">
         <v>12</v>
       </c>
       <c r="U26" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="V26" t="s">
         <v>1</v>
@@ -2569,19 +2647,19 @@
     </row>
     <row r="27" spans="1:25">
       <c r="A27" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B27" t="s">
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D27" t="s">
-        <v>81</v>
+        <v>16</v>
       </c>
       <c r="E27" s="2">
-        <v>46078</v>
+        <v>46050</v>
       </c>
       <c r="F27" s="3">
         <v>1</v>
@@ -2596,7 +2674,7 @@
         <v>4</v>
       </c>
       <c r="J27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="K27" t="s">
         <v>6</v>
@@ -2623,7 +2701,7 @@
         <v>1</v>
       </c>
       <c r="S27" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T27" t="s">
         <v>12</v>
@@ -2646,34 +2724,34 @@
     </row>
     <row r="28" spans="1:25">
       <c r="A28" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B28" t="s">
         <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>41</v>
+        <v>80</v>
       </c>
       <c r="D28" t="s">
-        <v>42</v>
+        <v>84</v>
       </c>
       <c r="E28" s="2">
-        <v>46078</v>
+        <v>46050</v>
       </c>
       <c r="F28" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G28" s="3">
         <v>0</v>
       </c>
       <c r="H28" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I28" t="s">
         <v>4</v>
       </c>
       <c r="J28" t="s">
-        <v>43</v>
+        <v>82</v>
       </c>
       <c r="K28" t="s">
         <v>6</v>
@@ -2688,7 +2766,7 @@
         <v>1</v>
       </c>
       <c r="O28" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="P28" t="s">
         <v>10</v>
@@ -2700,13 +2778,13 @@
         <v>1</v>
       </c>
       <c r="S28" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T28" t="s">
         <v>12</v>
       </c>
       <c r="U28" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="V28" t="s">
         <v>1</v>
@@ -2723,19 +2801,19 @@
     </row>
     <row r="29" spans="1:25">
       <c r="A29" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B29" t="s">
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>31</v>
+        <v>96</v>
       </c>
       <c r="D29" t="s">
-        <v>68</v>
+        <v>97</v>
       </c>
       <c r="E29" s="2">
-        <v>46063</v>
+        <v>46050</v>
       </c>
       <c r="F29" s="3">
         <v>1</v>
@@ -2750,7 +2828,7 @@
         <v>4</v>
       </c>
       <c r="J29" t="s">
-        <v>33</v>
+        <v>98</v>
       </c>
       <c r="K29" t="s">
         <v>6</v>
@@ -2765,7 +2843,7 @@
         <v>1</v>
       </c>
       <c r="O29" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="P29" t="s">
         <v>10</v>
@@ -2783,7 +2861,7 @@
         <v>12</v>
       </c>
       <c r="U29" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="V29" t="s">
         <v>1</v>
@@ -2800,19 +2878,19 @@
     </row>
     <row r="30" spans="1:25">
       <c r="A30" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B30" t="s">
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="D30" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E30" s="2">
-        <v>46063</v>
+        <v>46050</v>
       </c>
       <c r="F30" s="3">
         <v>1</v>
@@ -2827,7 +2905,7 @@
         <v>4</v>
       </c>
       <c r="J30" t="s">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="K30" t="s">
         <v>6</v>
@@ -2842,7 +2920,7 @@
         <v>1</v>
       </c>
       <c r="O30" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="P30" t="s">
         <v>10</v>
@@ -2860,7 +2938,7 @@
         <v>12</v>
       </c>
       <c r="U30" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="V30" t="s">
         <v>1</v>
@@ -2877,19 +2955,19 @@
     </row>
     <row r="31" spans="1:25">
       <c r="A31" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B31" t="s">
         <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="D31" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="E31" s="2">
-        <v>46065</v>
+        <v>46050</v>
       </c>
       <c r="F31" s="3">
         <v>1</v>
@@ -2904,7 +2982,7 @@
         <v>4</v>
       </c>
       <c r="J31" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="K31" t="s">
         <v>6</v>
@@ -2919,7 +2997,7 @@
         <v>1</v>
       </c>
       <c r="O31" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="P31" t="s">
         <v>10</v>
@@ -2937,7 +3015,7 @@
         <v>12</v>
       </c>
       <c r="U31" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="V31" t="s">
         <v>1</v>
@@ -2954,19 +3032,19 @@
     </row>
     <row r="32" spans="1:25">
       <c r="A32" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B32" t="s">
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>99</v>
+        <v>47</v>
       </c>
       <c r="D32" t="s">
-        <v>100</v>
+        <v>48</v>
       </c>
       <c r="E32" s="2">
-        <v>46066</v>
+        <v>46092</v>
       </c>
       <c r="F32" s="3">
         <v>1</v>
@@ -2981,7 +3059,7 @@
         <v>4</v>
       </c>
       <c r="J32" t="s">
-        <v>101</v>
+        <v>49</v>
       </c>
       <c r="K32" t="s">
         <v>6</v>
@@ -2996,7 +3074,7 @@
         <v>1</v>
       </c>
       <c r="O32" t="s">
-        <v>75</v>
+        <v>23</v>
       </c>
       <c r="P32" t="s">
         <v>10</v>
@@ -3014,7 +3092,7 @@
         <v>12</v>
       </c>
       <c r="U32" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="V32" t="s">
         <v>1</v>
@@ -3031,19 +3109,19 @@
     </row>
     <row r="33" spans="1:25">
       <c r="A33" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B33" t="s">
         <v>1</v>
       </c>
       <c r="C33" t="s">
-        <v>103</v>
+        <v>47</v>
       </c>
       <c r="D33" t="s">
-        <v>104</v>
+        <v>48</v>
       </c>
       <c r="E33" s="2">
-        <v>46050</v>
+        <v>46092</v>
       </c>
       <c r="F33" s="3">
         <v>1</v>
@@ -3058,7 +3136,7 @@
         <v>4</v>
       </c>
       <c r="J33" t="s">
-        <v>105</v>
+        <v>49</v>
       </c>
       <c r="K33" t="s">
         <v>6</v>
@@ -3073,7 +3151,7 @@
         <v>1</v>
       </c>
       <c r="O33" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="P33" t="s">
         <v>10</v>
@@ -3085,7 +3163,7 @@
         <v>1</v>
       </c>
       <c r="S33" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T33" t="s">
         <v>12</v>
@@ -3108,35 +3186,35 @@
     </row>
     <row r="34" spans="1:25">
       <c r="A34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B34" t="s">
         <v>1</v>
       </c>
       <c r="C34" t="s">
+        <v>105</v>
+      </c>
+      <c r="D34" t="s">
+        <v>3</v>
+      </c>
+      <c r="E34" s="2">
+        <v>46094</v>
+      </c>
+      <c r="F34" s="3">
+        <v>1</v>
+      </c>
+      <c r="G34" s="3">
+        <v>0</v>
+      </c>
+      <c r="H34" s="3">
+        <v>1</v>
+      </c>
+      <c r="I34" t="s">
+        <v>4</v>
+      </c>
+      <c r="J34" t="s">
         <v>106</v>
       </c>
-      <c r="D34" t="s">
-        <v>47</v>
-      </c>
-      <c r="E34" s="2">
-        <v>46050</v>
-      </c>
-      <c r="F34" s="3">
-        <v>2</v>
-      </c>
-      <c r="G34" s="3">
-        <v>1</v>
-      </c>
-      <c r="H34" s="3">
-        <v>1</v>
-      </c>
-      <c r="I34" t="s">
-        <v>4</v>
-      </c>
-      <c r="J34" t="s">
-        <v>107</v>
-      </c>
       <c r="K34" t="s">
         <v>6</v>
       </c>
@@ -3150,13 +3228,13 @@
         <v>1</v>
       </c>
       <c r="O34" t="s">
-        <v>54</v>
+        <v>9</v>
       </c>
       <c r="P34" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="Q34" t="s">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="R34" t="s">
         <v>1</v>
@@ -3168,7 +3246,7 @@
         <v>12</v>
       </c>
       <c r="U34" t="s">
-        <v>23</v>
+        <v>78</v>
       </c>
       <c r="V34" t="s">
         <v>1</v>
@@ -3185,35 +3263,35 @@
     </row>
     <row r="35" spans="1:25">
       <c r="A35" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B35" t="s">
         <v>1</v>
       </c>
       <c r="C35" t="s">
+        <v>107</v>
+      </c>
+      <c r="D35" t="s">
+        <v>43</v>
+      </c>
+      <c r="E35" s="2">
+        <v>46094</v>
+      </c>
+      <c r="F35" s="3">
+        <v>1</v>
+      </c>
+      <c r="G35" s="3">
+        <v>0</v>
+      </c>
+      <c r="H35" s="3">
+        <v>1</v>
+      </c>
+      <c r="I35" t="s">
+        <v>4</v>
+      </c>
+      <c r="J35" t="s">
         <v>108</v>
       </c>
-      <c r="D35" t="s">
-        <v>47</v>
-      </c>
-      <c r="E35" s="2">
-        <v>46050</v>
-      </c>
-      <c r="F35" s="3">
-        <v>1</v>
-      </c>
-      <c r="G35" s="3">
-        <v>0</v>
-      </c>
-      <c r="H35" s="3">
-        <v>1</v>
-      </c>
-      <c r="I35" t="s">
-        <v>4</v>
-      </c>
-      <c r="J35" t="s">
-        <v>109</v>
-      </c>
       <c r="K35" t="s">
         <v>6</v>
       </c>
@@ -3227,25 +3305,25 @@
         <v>1</v>
       </c>
       <c r="O35" t="s">
-        <v>54</v>
+        <v>9</v>
       </c>
       <c r="P35" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="Q35" t="s">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="R35" t="s">
         <v>1</v>
       </c>
       <c r="S35" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T35" t="s">
         <v>12</v>
       </c>
       <c r="U35" t="s">
-        <v>23</v>
+        <v>78</v>
       </c>
       <c r="V35" t="s">
         <v>1</v>
@@ -3262,19 +3340,19 @@
     </row>
     <row r="36" spans="1:25">
       <c r="A36" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B36" t="s">
         <v>1</v>
       </c>
       <c r="C36" t="s">
-        <v>99</v>
+        <v>74</v>
       </c>
       <c r="D36" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
       <c r="E36" s="2">
-        <v>46050</v>
+        <v>46094</v>
       </c>
       <c r="F36" s="3">
         <v>1</v>
@@ -3289,7 +3367,7 @@
         <v>4</v>
       </c>
       <c r="J36" t="s">
-        <v>101</v>
+        <v>76</v>
       </c>
       <c r="K36" t="s">
         <v>6</v>
@@ -3304,25 +3382,25 @@
         <v>1</v>
       </c>
       <c r="O36" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="P36" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="Q36" t="s">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="R36" t="s">
         <v>1</v>
       </c>
       <c r="S36" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T36" t="s">
         <v>12</v>
       </c>
       <c r="U36" t="s">
-        <v>1</v>
+        <v>78</v>
       </c>
       <c r="V36" t="s">
         <v>1</v>
@@ -3339,19 +3417,19 @@
     </row>
     <row r="37" spans="1:25">
       <c r="A37" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B37" t="s">
         <v>1</v>
       </c>
       <c r="C37" t="s">
+        <v>109</v>
+      </c>
+      <c r="D37" t="s">
         <v>110</v>
       </c>
-      <c r="D37" t="s">
-        <v>75</v>
-      </c>
       <c r="E37" s="2">
-        <v>46050</v>
+        <v>46094</v>
       </c>
       <c r="F37" s="3">
         <v>1</v>
@@ -3381,25 +3459,25 @@
         <v>1</v>
       </c>
       <c r="O37" t="s">
-        <v>44</v>
+        <v>77</v>
       </c>
       <c r="P37" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="Q37" t="s">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="R37" t="s">
         <v>1</v>
       </c>
       <c r="S37" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T37" t="s">
         <v>12</v>
       </c>
       <c r="U37" t="s">
-        <v>1</v>
+        <v>78</v>
       </c>
       <c r="V37" t="s">
         <v>1</v>
@@ -3422,13 +3500,13 @@
         <v>1</v>
       </c>
       <c r="C38" t="s">
-        <v>113</v>
+        <v>47</v>
       </c>
       <c r="D38" t="s">
-        <v>3</v>
+        <v>52</v>
       </c>
       <c r="E38" s="2">
-        <v>46044</v>
+        <v>46092</v>
       </c>
       <c r="F38" s="3">
         <v>1</v>
@@ -3443,7 +3521,7 @@
         <v>4</v>
       </c>
       <c r="J38" t="s">
-        <v>114</v>
+        <v>49</v>
       </c>
       <c r="K38" t="s">
         <v>6</v>
@@ -3458,7 +3536,7 @@
         <v>1</v>
       </c>
       <c r="O38" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="P38" t="s">
         <v>10</v>
@@ -3470,13 +3548,13 @@
         <v>1</v>
       </c>
       <c r="S38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T38" t="s">
         <v>12</v>
       </c>
       <c r="U38" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="V38" t="s">
         <v>1</v>
@@ -3488,6 +3566,930 @@
         <v>1</v>
       </c>
       <c r="Y38" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="39" spans="1:25">
+      <c r="A39" t="s">
+        <v>113</v>
+      </c>
+      <c r="B39" t="s">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>114</v>
+      </c>
+      <c r="D39" t="s">
+        <v>7</v>
+      </c>
+      <c r="E39" s="2">
+        <v>46093</v>
+      </c>
+      <c r="F39" s="3">
+        <v>1</v>
+      </c>
+      <c r="G39" s="3">
+        <v>0</v>
+      </c>
+      <c r="H39" s="3">
+        <v>1</v>
+      </c>
+      <c r="I39" t="s">
+        <v>4</v>
+      </c>
+      <c r="J39" t="s">
+        <v>115</v>
+      </c>
+      <c r="K39" t="s">
+        <v>6</v>
+      </c>
+      <c r="L39" t="s">
+        <v>7</v>
+      </c>
+      <c r="M39" t="s">
+        <v>8</v>
+      </c>
+      <c r="N39" t="s">
+        <v>116</v>
+      </c>
+      <c r="O39" t="s">
+        <v>117</v>
+      </c>
+      <c r="P39" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>11</v>
+      </c>
+      <c r="R39" t="s">
+        <v>1</v>
+      </c>
+      <c r="S39" s="3">
+        <v>1</v>
+      </c>
+      <c r="T39" t="s">
+        <v>12</v>
+      </c>
+      <c r="U39" t="s">
+        <v>13</v>
+      </c>
+      <c r="V39" t="s">
+        <v>1</v>
+      </c>
+      <c r="W39" t="s">
+        <v>1</v>
+      </c>
+      <c r="X39" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y39" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="40" spans="1:25">
+      <c r="A40" t="s">
+        <v>113</v>
+      </c>
+      <c r="B40" t="s">
+        <v>1</v>
+      </c>
+      <c r="C40" t="s">
+        <v>118</v>
+      </c>
+      <c r="D40" t="s">
+        <v>119</v>
+      </c>
+      <c r="E40" s="2">
+        <v>46093</v>
+      </c>
+      <c r="F40" s="3">
+        <v>1</v>
+      </c>
+      <c r="G40" s="3">
+        <v>0</v>
+      </c>
+      <c r="H40" s="3">
+        <v>1</v>
+      </c>
+      <c r="I40" t="s">
+        <v>4</v>
+      </c>
+      <c r="J40" t="s">
+        <v>120</v>
+      </c>
+      <c r="K40" t="s">
+        <v>6</v>
+      </c>
+      <c r="L40" t="s">
+        <v>7</v>
+      </c>
+      <c r="M40" t="s">
+        <v>8</v>
+      </c>
+      <c r="N40" t="s">
+        <v>116</v>
+      </c>
+      <c r="O40" t="s">
+        <v>117</v>
+      </c>
+      <c r="P40" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>11</v>
+      </c>
+      <c r="R40" t="s">
+        <v>1</v>
+      </c>
+      <c r="S40" s="3">
+        <v>1</v>
+      </c>
+      <c r="T40" t="s">
+        <v>12</v>
+      </c>
+      <c r="U40" t="s">
+        <v>13</v>
+      </c>
+      <c r="V40" t="s">
+        <v>1</v>
+      </c>
+      <c r="W40" t="s">
+        <v>1</v>
+      </c>
+      <c r="X40" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y40" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="41" spans="1:25">
+      <c r="A41" t="s">
+        <v>113</v>
+      </c>
+      <c r="B41" t="s">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>121</v>
+      </c>
+      <c r="D41" t="s">
+        <v>122</v>
+      </c>
+      <c r="E41" s="2">
+        <v>46093</v>
+      </c>
+      <c r="F41" s="3">
+        <v>1</v>
+      </c>
+      <c r="G41" s="3">
+        <v>0</v>
+      </c>
+      <c r="H41" s="3">
+        <v>1</v>
+      </c>
+      <c r="I41" t="s">
+        <v>4</v>
+      </c>
+      <c r="J41" t="s">
+        <v>123</v>
+      </c>
+      <c r="K41" t="s">
+        <v>6</v>
+      </c>
+      <c r="L41" t="s">
+        <v>7</v>
+      </c>
+      <c r="M41" t="s">
+        <v>8</v>
+      </c>
+      <c r="N41" t="s">
+        <v>1</v>
+      </c>
+      <c r="O41" t="s">
+        <v>124</v>
+      </c>
+      <c r="P41" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q41" t="s">
+        <v>11</v>
+      </c>
+      <c r="R41" t="s">
+        <v>1</v>
+      </c>
+      <c r="S41" s="3">
+        <v>1</v>
+      </c>
+      <c r="T41" t="s">
+        <v>12</v>
+      </c>
+      <c r="U41" t="s">
+        <v>13</v>
+      </c>
+      <c r="V41" t="s">
+        <v>1</v>
+      </c>
+      <c r="W41" t="s">
+        <v>1</v>
+      </c>
+      <c r="X41" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y41" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="42" spans="1:25">
+      <c r="A42" t="s">
+        <v>113</v>
+      </c>
+      <c r="B42" t="s">
+        <v>1</v>
+      </c>
+      <c r="C42" t="s">
+        <v>47</v>
+      </c>
+      <c r="D42" t="s">
+        <v>52</v>
+      </c>
+      <c r="E42" s="2">
+        <v>46093</v>
+      </c>
+      <c r="F42" s="3">
+        <v>1</v>
+      </c>
+      <c r="G42" s="3">
+        <v>0</v>
+      </c>
+      <c r="H42" s="3">
+        <v>1</v>
+      </c>
+      <c r="I42" t="s">
+        <v>4</v>
+      </c>
+      <c r="J42" t="s">
+        <v>49</v>
+      </c>
+      <c r="K42" t="s">
+        <v>6</v>
+      </c>
+      <c r="L42" t="s">
+        <v>7</v>
+      </c>
+      <c r="M42" t="s">
+        <v>8</v>
+      </c>
+      <c r="N42" t="s">
+        <v>1</v>
+      </c>
+      <c r="O42" t="s">
+        <v>23</v>
+      </c>
+      <c r="P42" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q42" t="s">
+        <v>11</v>
+      </c>
+      <c r="R42" t="s">
+        <v>1</v>
+      </c>
+      <c r="S42" s="3">
+        <v>1</v>
+      </c>
+      <c r="T42" t="s">
+        <v>12</v>
+      </c>
+      <c r="U42" t="s">
+        <v>13</v>
+      </c>
+      <c r="V42" t="s">
+        <v>1</v>
+      </c>
+      <c r="W42" t="s">
+        <v>1</v>
+      </c>
+      <c r="X42" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y42" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="43" spans="1:25">
+      <c r="A43" t="s">
+        <v>125</v>
+      </c>
+      <c r="B43" t="s">
+        <v>1</v>
+      </c>
+      <c r="C43" t="s">
+        <v>126</v>
+      </c>
+      <c r="D43" t="s">
+        <v>7</v>
+      </c>
+      <c r="E43" s="2">
+        <v>46086</v>
+      </c>
+      <c r="F43" s="3">
+        <v>2</v>
+      </c>
+      <c r="G43" s="3">
+        <v>0</v>
+      </c>
+      <c r="H43" s="3">
+        <v>2</v>
+      </c>
+      <c r="I43" t="s">
+        <v>4</v>
+      </c>
+      <c r="J43" t="s">
+        <v>127</v>
+      </c>
+      <c r="K43" t="s">
+        <v>6</v>
+      </c>
+      <c r="L43" t="s">
+        <v>7</v>
+      </c>
+      <c r="M43" t="s">
+        <v>8</v>
+      </c>
+      <c r="N43" t="s">
+        <v>1</v>
+      </c>
+      <c r="O43" t="s">
+        <v>117</v>
+      </c>
+      <c r="P43" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q43" t="s">
+        <v>11</v>
+      </c>
+      <c r="R43" t="s">
+        <v>1</v>
+      </c>
+      <c r="S43" s="3">
+        <v>2</v>
+      </c>
+      <c r="T43" t="s">
+        <v>12</v>
+      </c>
+      <c r="U43" t="s">
+        <v>13</v>
+      </c>
+      <c r="V43" t="s">
+        <v>1</v>
+      </c>
+      <c r="W43" t="s">
+        <v>1</v>
+      </c>
+      <c r="X43" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y43" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="44" spans="1:25">
+      <c r="A44" t="s">
+        <v>125</v>
+      </c>
+      <c r="B44" t="s">
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
+        <v>80</v>
+      </c>
+      <c r="D44" t="s">
+        <v>122</v>
+      </c>
+      <c r="E44" s="2">
+        <v>46086</v>
+      </c>
+      <c r="F44" s="3">
+        <v>2</v>
+      </c>
+      <c r="G44" s="3">
+        <v>0</v>
+      </c>
+      <c r="H44" s="3">
+        <v>2</v>
+      </c>
+      <c r="I44" t="s">
+        <v>4</v>
+      </c>
+      <c r="J44" t="s">
+        <v>82</v>
+      </c>
+      <c r="K44" t="s">
+        <v>6</v>
+      </c>
+      <c r="L44" t="s">
+        <v>7</v>
+      </c>
+      <c r="M44" t="s">
+        <v>8</v>
+      </c>
+      <c r="N44" t="s">
+        <v>1</v>
+      </c>
+      <c r="O44" t="s">
+        <v>23</v>
+      </c>
+      <c r="P44" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q44" t="s">
+        <v>11</v>
+      </c>
+      <c r="R44" t="s">
+        <v>1</v>
+      </c>
+      <c r="S44" s="3">
+        <v>2</v>
+      </c>
+      <c r="T44" t="s">
+        <v>12</v>
+      </c>
+      <c r="U44" t="s">
+        <v>13</v>
+      </c>
+      <c r="V44" t="s">
+        <v>1</v>
+      </c>
+      <c r="W44" t="s">
+        <v>1</v>
+      </c>
+      <c r="X44" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y44" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="45" spans="1:25">
+      <c r="A45" t="s">
+        <v>125</v>
+      </c>
+      <c r="B45" t="s">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>83</v>
+      </c>
+      <c r="D45" t="s">
+        <v>128</v>
+      </c>
+      <c r="E45" s="2">
+        <v>46086</v>
+      </c>
+      <c r="F45" s="3">
+        <v>1</v>
+      </c>
+      <c r="G45" s="3">
+        <v>0</v>
+      </c>
+      <c r="H45" s="3">
+        <v>1</v>
+      </c>
+      <c r="I45" t="s">
+        <v>4</v>
+      </c>
+      <c r="J45" t="s">
+        <v>85</v>
+      </c>
+      <c r="K45" t="s">
+        <v>6</v>
+      </c>
+      <c r="L45" t="s">
+        <v>7</v>
+      </c>
+      <c r="M45" t="s">
+        <v>8</v>
+      </c>
+      <c r="N45" t="s">
+        <v>1</v>
+      </c>
+      <c r="O45" t="s">
+        <v>23</v>
+      </c>
+      <c r="P45" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q45" t="s">
+        <v>11</v>
+      </c>
+      <c r="R45" t="s">
+        <v>1</v>
+      </c>
+      <c r="S45" s="3">
+        <v>1</v>
+      </c>
+      <c r="T45" t="s">
+        <v>12</v>
+      </c>
+      <c r="U45" t="s">
+        <v>13</v>
+      </c>
+      <c r="V45" t="s">
+        <v>1</v>
+      </c>
+      <c r="W45" t="s">
+        <v>1</v>
+      </c>
+      <c r="X45" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y45" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="46" spans="1:25">
+      <c r="A46" t="s">
+        <v>125</v>
+      </c>
+      <c r="B46" t="s">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
+        <v>129</v>
+      </c>
+      <c r="D46" t="s">
+        <v>130</v>
+      </c>
+      <c r="E46" s="2">
+        <v>46086</v>
+      </c>
+      <c r="F46" s="3">
+        <v>1</v>
+      </c>
+      <c r="G46" s="3">
+        <v>0</v>
+      </c>
+      <c r="H46" s="3">
+        <v>1</v>
+      </c>
+      <c r="I46" t="s">
+        <v>4</v>
+      </c>
+      <c r="J46" t="s">
+        <v>131</v>
+      </c>
+      <c r="K46" t="s">
+        <v>6</v>
+      </c>
+      <c r="L46" t="s">
+        <v>7</v>
+      </c>
+      <c r="M46" t="s">
+        <v>8</v>
+      </c>
+      <c r="N46" t="s">
+        <v>1</v>
+      </c>
+      <c r="O46" t="s">
+        <v>23</v>
+      </c>
+      <c r="P46" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q46" t="s">
+        <v>11</v>
+      </c>
+      <c r="R46" t="s">
+        <v>1</v>
+      </c>
+      <c r="S46" s="3">
+        <v>1</v>
+      </c>
+      <c r="T46" t="s">
+        <v>12</v>
+      </c>
+      <c r="U46" t="s">
+        <v>13</v>
+      </c>
+      <c r="V46" t="s">
+        <v>1</v>
+      </c>
+      <c r="W46" t="s">
+        <v>1</v>
+      </c>
+      <c r="X46" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y46" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="47" spans="1:25">
+      <c r="A47" t="s">
+        <v>125</v>
+      </c>
+      <c r="B47" t="s">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>99</v>
+      </c>
+      <c r="D47" t="s">
+        <v>97</v>
+      </c>
+      <c r="E47" s="2">
+        <v>46086</v>
+      </c>
+      <c r="F47" s="3">
+        <v>1</v>
+      </c>
+      <c r="G47" s="3">
+        <v>0</v>
+      </c>
+      <c r="H47" s="3">
+        <v>1</v>
+      </c>
+      <c r="I47" t="s">
+        <v>4</v>
+      </c>
+      <c r="J47" t="s">
+        <v>101</v>
+      </c>
+      <c r="K47" t="s">
+        <v>6</v>
+      </c>
+      <c r="L47" t="s">
+        <v>7</v>
+      </c>
+      <c r="M47" t="s">
+        <v>8</v>
+      </c>
+      <c r="N47" t="s">
+        <v>1</v>
+      </c>
+      <c r="O47" t="s">
+        <v>23</v>
+      </c>
+      <c r="P47" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q47" t="s">
+        <v>11</v>
+      </c>
+      <c r="R47" t="s">
+        <v>1</v>
+      </c>
+      <c r="S47" s="3">
+        <v>1</v>
+      </c>
+      <c r="T47" t="s">
+        <v>12</v>
+      </c>
+      <c r="U47" t="s">
+        <v>13</v>
+      </c>
+      <c r="V47" t="s">
+        <v>1</v>
+      </c>
+      <c r="W47" t="s">
+        <v>1</v>
+      </c>
+      <c r="X47" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y47" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="48" spans="1:25">
+      <c r="A48" t="s">
+        <v>125</v>
+      </c>
+      <c r="B48" t="s">
+        <v>1</v>
+      </c>
+      <c r="C48" t="s">
+        <v>132</v>
+      </c>
+      <c r="D48" t="s">
+        <v>52</v>
+      </c>
+      <c r="E48" s="2">
+        <v>46086</v>
+      </c>
+      <c r="F48" s="3">
+        <v>1</v>
+      </c>
+      <c r="G48" s="3">
+        <v>0</v>
+      </c>
+      <c r="H48" s="3">
+        <v>1</v>
+      </c>
+      <c r="I48" t="s">
+        <v>4</v>
+      </c>
+      <c r="J48" t="s">
+        <v>133</v>
+      </c>
+      <c r="K48" t="s">
+        <v>6</v>
+      </c>
+      <c r="L48" t="s">
+        <v>7</v>
+      </c>
+      <c r="M48" t="s">
+        <v>8</v>
+      </c>
+      <c r="N48" t="s">
+        <v>1</v>
+      </c>
+      <c r="O48" t="s">
+        <v>23</v>
+      </c>
+      <c r="P48" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q48" t="s">
+        <v>11</v>
+      </c>
+      <c r="R48" t="s">
+        <v>1</v>
+      </c>
+      <c r="S48" s="3">
+        <v>1</v>
+      </c>
+      <c r="T48" t="s">
+        <v>12</v>
+      </c>
+      <c r="U48" t="s">
+        <v>13</v>
+      </c>
+      <c r="V48" t="s">
+        <v>1</v>
+      </c>
+      <c r="W48" t="s">
+        <v>1</v>
+      </c>
+      <c r="X48" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y48" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="49" spans="1:25">
+      <c r="A49" t="s">
+        <v>134</v>
+      </c>
+      <c r="B49" t="s">
+        <v>1</v>
+      </c>
+      <c r="C49" t="s">
+        <v>135</v>
+      </c>
+      <c r="D49" t="s">
+        <v>136</v>
+      </c>
+      <c r="E49" s="2">
+        <v>46059</v>
+      </c>
+      <c r="F49" s="3">
+        <v>1</v>
+      </c>
+      <c r="G49" s="3">
+        <v>0</v>
+      </c>
+      <c r="H49" s="3">
+        <v>1</v>
+      </c>
+      <c r="I49" t="s">
+        <v>4</v>
+      </c>
+      <c r="J49" t="s">
+        <v>137</v>
+      </c>
+      <c r="K49" t="s">
+        <v>6</v>
+      </c>
+      <c r="L49" t="s">
+        <v>7</v>
+      </c>
+      <c r="M49" t="s">
+        <v>8</v>
+      </c>
+      <c r="N49" t="s">
+        <v>1</v>
+      </c>
+      <c r="O49" t="s">
+        <v>30</v>
+      </c>
+      <c r="P49" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q49" t="s">
+        <v>11</v>
+      </c>
+      <c r="R49" t="s">
+        <v>1</v>
+      </c>
+      <c r="S49" s="3">
+        <v>0</v>
+      </c>
+      <c r="T49" t="s">
+        <v>12</v>
+      </c>
+      <c r="U49" t="s">
+        <v>1</v>
+      </c>
+      <c r="V49" t="s">
+        <v>1</v>
+      </c>
+      <c r="W49" t="s">
+        <v>1</v>
+      </c>
+      <c r="X49" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y49" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="50" spans="1:25">
+      <c r="A50" t="s">
+        <v>138</v>
+      </c>
+      <c r="B50" t="s">
+        <v>1</v>
+      </c>
+      <c r="C50" t="s">
+        <v>139</v>
+      </c>
+      <c r="D50" t="s">
+        <v>119</v>
+      </c>
+      <c r="E50" s="2">
+        <v>46064</v>
+      </c>
+      <c r="F50" s="3">
+        <v>1</v>
+      </c>
+      <c r="G50" s="3">
+        <v>0</v>
+      </c>
+      <c r="H50" s="3">
+        <v>1</v>
+      </c>
+      <c r="I50" t="s">
+        <v>4</v>
+      </c>
+      <c r="J50" t="s">
+        <v>140</v>
+      </c>
+      <c r="K50" t="s">
+        <v>6</v>
+      </c>
+      <c r="L50" t="s">
+        <v>7</v>
+      </c>
+      <c r="M50" t="s">
+        <v>8</v>
+      </c>
+      <c r="N50" t="s">
+        <v>1</v>
+      </c>
+      <c r="O50" t="s">
+        <v>30</v>
+      </c>
+      <c r="P50" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q50" t="s">
+        <v>11</v>
+      </c>
+      <c r="R50" t="s">
+        <v>1</v>
+      </c>
+      <c r="S50" s="3">
+        <v>0</v>
+      </c>
+      <c r="T50" t="s">
+        <v>12</v>
+      </c>
+      <c r="U50" t="s">
+        <v>1</v>
+      </c>
+      <c r="V50" t="s">
+        <v>1</v>
+      </c>
+      <c r="W50" t="s">
+        <v>1</v>
+      </c>
+      <c r="X50" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y50" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance semi-finished auto-dispatch logic and implement dedicated shortage summary page
</commit_message>
<xml_diff>
--- a/Newdata/已撥缺料.XLSX
+++ b/Newdata/已撥缺料.XLSX
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1065" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1045" uniqueCount="158">
   <si>
     <t>200006482</t>
   </si>
@@ -221,15 +221,6 @@
   </si>
   <si>
     <t>0107</t>
-  </si>
-  <si>
-    <t>200006573</t>
-  </si>
-  <si>
-    <t>3154001348A1</t>
-  </si>
-  <si>
-    <t>主軸前蓋_INC-H-90</t>
   </si>
   <si>
     <t>200006578</t>
@@ -598,7 +589,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:Y53"/>
+  <dimension ref="A1:Y52"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="11" customWidth="1"/>
@@ -630,79 +621,79 @@
   <sheetData>
     <row r="1" spans="1:25">
       <c r="A1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="G1" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="J1" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="K1" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="L1" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="S1" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="V1" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="2" spans="1:25">
@@ -2179,10 +2170,10 @@
         <v>71</v>
       </c>
       <c r="D21" t="s">
-        <v>16</v>
+        <v>72</v>
       </c>
       <c r="E21" s="2">
-        <v>46167</v>
+        <v>46106</v>
       </c>
       <c r="F21" s="3">
         <v>1</v>
@@ -2197,7 +2188,7 @@
         <v>4</v>
       </c>
       <c r="J21" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K21" t="s">
         <v>6</v>
@@ -2212,13 +2203,13 @@
         <v>1</v>
       </c>
       <c r="O21" t="s">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="P21" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="Q21" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="R21" t="s">
         <v>1</v>
@@ -2230,7 +2221,7 @@
         <v>12</v>
       </c>
       <c r="U21" t="s">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="V21" t="s">
         <v>1</v>
@@ -2247,7 +2238,7 @@
     </row>
     <row r="22" spans="1:25">
       <c r="A22" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B22" t="s">
         <v>1</v>
@@ -2256,7 +2247,7 @@
         <v>74</v>
       </c>
       <c r="D22" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="E22" s="2">
         <v>46106</v>
@@ -2274,7 +2265,7 @@
         <v>4</v>
       </c>
       <c r="J22" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K22" t="s">
         <v>6</v>
@@ -2289,7 +2280,7 @@
         <v>1</v>
       </c>
       <c r="O22" t="s">
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="P22" t="s">
         <v>29</v>
@@ -2307,7 +2298,7 @@
         <v>12</v>
       </c>
       <c r="U22" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="V22" t="s">
         <v>1</v>
@@ -2324,16 +2315,16 @@
     </row>
     <row r="23" spans="1:25">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B23" t="s">
         <v>1</v>
       </c>
       <c r="C23" t="s">
+        <v>76</v>
+      </c>
+      <c r="D23" t="s">
         <v>77</v>
-      </c>
-      <c r="D23" t="s">
-        <v>45</v>
       </c>
       <c r="E23" s="2">
         <v>46106</v>
@@ -2366,7 +2357,7 @@
         <v>1</v>
       </c>
       <c r="O23" t="s">
-        <v>9</v>
+        <v>79</v>
       </c>
       <c r="P23" t="s">
         <v>29</v>
@@ -2378,13 +2369,13 @@
         <v>1</v>
       </c>
       <c r="S23" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T23" t="s">
         <v>12</v>
       </c>
       <c r="U23" t="s">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="V23" t="s">
         <v>1</v>
@@ -2401,16 +2392,16 @@
     </row>
     <row r="24" spans="1:25">
       <c r="A24" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B24" t="s">
         <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D24" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E24" s="2">
         <v>46106</v>
@@ -2428,7 +2419,7 @@
         <v>4</v>
       </c>
       <c r="J24" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K24" t="s">
         <v>6</v>
@@ -2443,7 +2434,7 @@
         <v>1</v>
       </c>
       <c r="O24" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="P24" t="s">
         <v>29</v>
@@ -2478,16 +2469,16 @@
     </row>
     <row r="25" spans="1:25">
       <c r="A25" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B25" t="s">
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D25" t="s">
-        <v>84</v>
+        <v>54</v>
       </c>
       <c r="E25" s="2">
         <v>46106</v>
@@ -2520,7 +2511,7 @@
         <v>1</v>
       </c>
       <c r="O25" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="P25" t="s">
         <v>29</v>
@@ -2555,7 +2546,7 @@
     </row>
     <row r="26" spans="1:25">
       <c r="A26" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="B26" t="s">
         <v>1</v>
@@ -2564,10 +2555,10 @@
         <v>87</v>
       </c>
       <c r="D26" t="s">
-        <v>54</v>
+        <v>88</v>
       </c>
       <c r="E26" s="2">
-        <v>46106</v>
+        <v>46097</v>
       </c>
       <c r="F26" s="3">
         <v>1</v>
@@ -2582,7 +2573,7 @@
         <v>4</v>
       </c>
       <c r="J26" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K26" t="s">
         <v>6</v>
@@ -2597,7 +2588,7 @@
         <v>1</v>
       </c>
       <c r="O26" t="s">
-        <v>86</v>
+        <v>48</v>
       </c>
       <c r="P26" t="s">
         <v>29</v>
@@ -2615,7 +2606,7 @@
         <v>12</v>
       </c>
       <c r="U26" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="V26" t="s">
         <v>1</v>
@@ -2632,19 +2623,19 @@
     </row>
     <row r="27" spans="1:25">
       <c r="A27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B27" t="s">
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D27" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E27" s="2">
-        <v>46097</v>
+        <v>46161</v>
       </c>
       <c r="F27" s="3">
         <v>1</v>
@@ -2659,7 +2650,7 @@
         <v>4</v>
       </c>
       <c r="J27" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K27" t="s">
         <v>6</v>
@@ -2674,7 +2665,7 @@
         <v>1</v>
       </c>
       <c r="O27" t="s">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="P27" t="s">
         <v>29</v>
@@ -2686,7 +2677,7 @@
         <v>1</v>
       </c>
       <c r="S27" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T27" t="s">
         <v>12</v>
@@ -2709,7 +2700,7 @@
     </row>
     <row r="28" spans="1:25">
       <c r="A28" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B28" t="s">
         <v>1</v>
@@ -2718,7 +2709,7 @@
         <v>94</v>
       </c>
       <c r="D28" t="s">
-        <v>95</v>
+        <v>27</v>
       </c>
       <c r="E28" s="2">
         <v>46161</v>
@@ -2736,7 +2727,7 @@
         <v>4</v>
       </c>
       <c r="J28" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K28" t="s">
         <v>6</v>
@@ -2786,7 +2777,7 @@
     </row>
     <row r="29" spans="1:25">
       <c r="A29" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B29" t="s">
         <v>1</v>
@@ -2795,7 +2786,7 @@
         <v>97</v>
       </c>
       <c r="D29" t="s">
-        <v>27</v>
+        <v>98</v>
       </c>
       <c r="E29" s="2">
         <v>46161</v>
@@ -2813,7 +2804,7 @@
         <v>4</v>
       </c>
       <c r="J29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K29" t="s">
         <v>6</v>
@@ -2863,19 +2854,19 @@
     </row>
     <row r="30" spans="1:25">
       <c r="A30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B30" t="s">
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D30" t="s">
-        <v>101</v>
+        <v>79</v>
       </c>
       <c r="E30" s="2">
-        <v>46161</v>
+        <v>46153</v>
       </c>
       <c r="F30" s="3">
         <v>1</v>
@@ -2905,7 +2896,7 @@
         <v>1</v>
       </c>
       <c r="O30" t="s">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="P30" t="s">
         <v>29</v>
@@ -2949,10 +2940,10 @@
         <v>104</v>
       </c>
       <c r="D31" t="s">
-        <v>82</v>
+        <v>39</v>
       </c>
       <c r="E31" s="2">
-        <v>46153</v>
+        <v>46134</v>
       </c>
       <c r="F31" s="3">
         <v>1</v>
@@ -2982,7 +2973,7 @@
         <v>1</v>
       </c>
       <c r="O31" t="s">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="P31" t="s">
         <v>29</v>
@@ -3023,13 +3014,13 @@
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="D32" t="s">
         <v>39</v>
       </c>
       <c r="E32" s="2">
-        <v>46134</v>
+        <v>46136</v>
       </c>
       <c r="F32" s="3">
         <v>1</v>
@@ -3044,7 +3035,7 @@
         <v>4</v>
       </c>
       <c r="J32" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="K32" t="s">
         <v>6</v>
@@ -3094,19 +3085,19 @@
     </row>
     <row r="33" spans="1:25">
       <c r="A33" t="s">
+        <v>107</v>
+      </c>
+      <c r="B33" t="s">
+        <v>1</v>
+      </c>
+      <c r="C33" t="s">
+        <v>108</v>
+      </c>
+      <c r="D33" t="s">
         <v>109</v>
       </c>
-      <c r="B33" t="s">
-        <v>1</v>
-      </c>
-      <c r="C33" t="s">
-        <v>107</v>
-      </c>
-      <c r="D33" t="s">
-        <v>39</v>
-      </c>
       <c r="E33" s="2">
-        <v>46136</v>
+        <v>46150</v>
       </c>
       <c r="F33" s="3">
         <v>1</v>
@@ -3121,7 +3112,7 @@
         <v>4</v>
       </c>
       <c r="J33" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K33" t="s">
         <v>6</v>
@@ -3136,7 +3127,7 @@
         <v>1</v>
       </c>
       <c r="O33" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P33" t="s">
         <v>29</v>
@@ -3154,7 +3145,7 @@
         <v>12</v>
       </c>
       <c r="U33" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="V33" t="s">
         <v>1</v>
@@ -3171,7 +3162,7 @@
     </row>
     <row r="34" spans="1:25">
       <c r="A34" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B34" t="s">
         <v>1</v>
@@ -3186,10 +3177,10 @@
         <v>46150</v>
       </c>
       <c r="F34" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G34" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H34" s="3">
         <v>1</v>
@@ -3213,7 +3204,7 @@
         <v>1</v>
       </c>
       <c r="O34" t="s">
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="P34" t="s">
         <v>29</v>
@@ -3225,13 +3216,13 @@
         <v>1</v>
       </c>
       <c r="S34" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T34" t="s">
         <v>12</v>
       </c>
       <c r="U34" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="V34" t="s">
         <v>1</v>
@@ -3248,25 +3239,25 @@
     </row>
     <row r="35" spans="1:25">
       <c r="A35" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B35" t="s">
         <v>1</v>
       </c>
       <c r="C35" t="s">
-        <v>114</v>
+        <v>91</v>
       </c>
       <c r="D35" t="s">
-        <v>115</v>
+        <v>92</v>
       </c>
       <c r="E35" s="2">
-        <v>46150</v>
+        <v>46133</v>
       </c>
       <c r="F35" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G35" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H35" s="3">
         <v>1</v>
@@ -3275,7 +3266,7 @@
         <v>4</v>
       </c>
       <c r="J35" t="s">
-        <v>116</v>
+        <v>93</v>
       </c>
       <c r="K35" t="s">
         <v>6</v>
@@ -3290,7 +3281,7 @@
         <v>1</v>
       </c>
       <c r="O35" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="P35" t="s">
         <v>29</v>
@@ -3302,7 +3293,7 @@
         <v>1</v>
       </c>
       <c r="S35" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T35" t="s">
         <v>12</v>
@@ -3325,7 +3316,7 @@
     </row>
     <row r="36" spans="1:25">
       <c r="A36" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B36" t="s">
         <v>1</v>
@@ -3334,7 +3325,7 @@
         <v>94</v>
       </c>
       <c r="D36" t="s">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="E36" s="2">
         <v>46133</v>
@@ -3352,7 +3343,7 @@
         <v>4</v>
       </c>
       <c r="J36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K36" t="s">
         <v>6</v>
@@ -3402,19 +3393,19 @@
     </row>
     <row r="37" spans="1:25">
       <c r="A37" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B37" t="s">
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>97</v>
+        <v>33</v>
       </c>
       <c r="D37" t="s">
-        <v>118</v>
+        <v>34</v>
       </c>
       <c r="E37" s="2">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="F37" s="3">
         <v>1</v>
@@ -3429,7 +3420,7 @@
         <v>4</v>
       </c>
       <c r="J37" t="s">
-        <v>98</v>
+        <v>35</v>
       </c>
       <c r="K37" t="s">
         <v>6</v>
@@ -3444,7 +3435,7 @@
         <v>1</v>
       </c>
       <c r="O37" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="P37" t="s">
         <v>29</v>
@@ -3479,35 +3470,35 @@
     </row>
     <row r="38" spans="1:25">
       <c r="A38" t="s">
+        <v>117</v>
+      </c>
+      <c r="B38" t="s">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>118</v>
+      </c>
+      <c r="D38" t="s">
+        <v>79</v>
+      </c>
+      <c r="E38" s="2">
+        <v>46139</v>
+      </c>
+      <c r="F38" s="3">
+        <v>1</v>
+      </c>
+      <c r="G38" s="3">
+        <v>0</v>
+      </c>
+      <c r="H38" s="3">
+        <v>1</v>
+      </c>
+      <c r="I38" t="s">
+        <v>4</v>
+      </c>
+      <c r="J38" t="s">
         <v>119</v>
       </c>
-      <c r="B38" t="s">
-        <v>1</v>
-      </c>
-      <c r="C38" t="s">
-        <v>33</v>
-      </c>
-      <c r="D38" t="s">
-        <v>34</v>
-      </c>
-      <c r="E38" s="2">
-        <v>46134</v>
-      </c>
-      <c r="F38" s="3">
-        <v>1</v>
-      </c>
-      <c r="G38" s="3">
-        <v>0</v>
-      </c>
-      <c r="H38" s="3">
-        <v>1</v>
-      </c>
-      <c r="I38" t="s">
-        <v>4</v>
-      </c>
-      <c r="J38" t="s">
-        <v>35</v>
-      </c>
       <c r="K38" t="s">
         <v>6</v>
       </c>
@@ -3521,7 +3512,7 @@
         <v>1</v>
       </c>
       <c r="O38" t="s">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="P38" t="s">
         <v>29</v>
@@ -3556,16 +3547,16 @@
     </row>
     <row r="39" spans="1:25">
       <c r="A39" t="s">
+        <v>117</v>
+      </c>
+      <c r="B39" t="s">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
         <v>120</v>
       </c>
-      <c r="B39" t="s">
-        <v>1</v>
-      </c>
-      <c r="C39" t="s">
-        <v>121</v>
-      </c>
       <c r="D39" t="s">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="E39" s="2">
         <v>46139</v>
@@ -3583,7 +3574,7 @@
         <v>4</v>
       </c>
       <c r="J39" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="K39" t="s">
         <v>6</v>
@@ -3633,16 +3624,16 @@
     </row>
     <row r="40" spans="1:25">
       <c r="A40" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B40" t="s">
         <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D40" t="s">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="E40" s="2">
         <v>46139</v>
@@ -3660,7 +3651,7 @@
         <v>4</v>
       </c>
       <c r="J40" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K40" t="s">
         <v>6</v>
@@ -3710,16 +3701,16 @@
     </row>
     <row r="41" spans="1:25">
       <c r="A41" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B41" t="s">
         <v>1</v>
       </c>
       <c r="C41" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="D41" t="s">
-        <v>27</v>
+        <v>79</v>
       </c>
       <c r="E41" s="2">
         <v>46139</v>
@@ -3737,7 +3728,7 @@
         <v>4</v>
       </c>
       <c r="J41" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="K41" t="s">
         <v>6</v>
@@ -3787,16 +3778,16 @@
     </row>
     <row r="42" spans="1:25">
       <c r="A42" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B42" t="s">
         <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D42" t="s">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="E42" s="2">
         <v>46139</v>
@@ -3814,7 +3805,7 @@
         <v>4</v>
       </c>
       <c r="J42" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="K42" t="s">
         <v>6</v>
@@ -3864,16 +3855,16 @@
     </row>
     <row r="43" spans="1:25">
       <c r="A43" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B43" t="s">
         <v>1</v>
       </c>
       <c r="C43" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D43" t="s">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="E43" s="2">
         <v>46139</v>
@@ -3891,7 +3882,7 @@
         <v>4</v>
       </c>
       <c r="J43" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K43" t="s">
         <v>6</v>
@@ -3941,16 +3932,16 @@
     </row>
     <row r="44" spans="1:25">
       <c r="A44" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B44" t="s">
         <v>1</v>
       </c>
       <c r="C44" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="D44" t="s">
-        <v>27</v>
+        <v>79</v>
       </c>
       <c r="E44" s="2">
         <v>46139</v>
@@ -3968,7 +3959,7 @@
         <v>4</v>
       </c>
       <c r="J44" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="K44" t="s">
         <v>6</v>
@@ -4018,16 +4009,16 @@
     </row>
     <row r="45" spans="1:25">
       <c r="A45" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B45" t="s">
         <v>1</v>
       </c>
       <c r="C45" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D45" t="s">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="E45" s="2">
         <v>46139</v>
@@ -4045,7 +4036,7 @@
         <v>4</v>
       </c>
       <c r="J45" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="K45" t="s">
         <v>6</v>
@@ -4095,16 +4086,16 @@
     </row>
     <row r="46" spans="1:25">
       <c r="A46" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B46" t="s">
         <v>1</v>
       </c>
       <c r="C46" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D46" t="s">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="E46" s="2">
         <v>46139</v>
@@ -4122,7 +4113,7 @@
         <v>4</v>
       </c>
       <c r="J46" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K46" t="s">
         <v>6</v>
@@ -4172,16 +4163,16 @@
     </row>
     <row r="47" spans="1:25">
       <c r="A47" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B47" t="s">
         <v>1</v>
       </c>
       <c r="C47" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="D47" t="s">
-        <v>27</v>
+        <v>79</v>
       </c>
       <c r="E47" s="2">
         <v>46139</v>
@@ -4199,7 +4190,7 @@
         <v>4</v>
       </c>
       <c r="J47" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="K47" t="s">
         <v>6</v>
@@ -4249,16 +4240,16 @@
     </row>
     <row r="48" spans="1:25">
       <c r="A48" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B48" t="s">
         <v>1</v>
       </c>
       <c r="C48" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D48" t="s">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="E48" s="2">
         <v>46139</v>
@@ -4276,7 +4267,7 @@
         <v>4</v>
       </c>
       <c r="J48" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="K48" t="s">
         <v>6</v>
@@ -4326,16 +4317,16 @@
     </row>
     <row r="49" spans="1:25">
       <c r="A49" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B49" t="s">
         <v>1</v>
       </c>
       <c r="C49" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D49" t="s">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="E49" s="2">
         <v>46139</v>
@@ -4353,7 +4344,7 @@
         <v>4</v>
       </c>
       <c r="J49" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K49" t="s">
         <v>6</v>
@@ -4403,19 +4394,19 @@
     </row>
     <row r="50" spans="1:25">
       <c r="A50" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B50" t="s">
         <v>1</v>
       </c>
       <c r="C50" t="s">
-        <v>125</v>
+        <v>26</v>
       </c>
       <c r="D50" t="s">
         <v>27</v>
       </c>
       <c r="E50" s="2">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="F50" s="3">
         <v>1</v>
@@ -4430,7 +4421,7 @@
         <v>4</v>
       </c>
       <c r="J50" t="s">
-        <v>126</v>
+        <v>28</v>
       </c>
       <c r="K50" t="s">
         <v>6</v>
@@ -4445,7 +4436,7 @@
         <v>1</v>
       </c>
       <c r="O50" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="P50" t="s">
         <v>29</v>
@@ -4480,35 +4471,35 @@
     </row>
     <row r="51" spans="1:25">
       <c r="A51" t="s">
+        <v>128</v>
+      </c>
+      <c r="B51" t="s">
+        <v>1</v>
+      </c>
+      <c r="C51" t="s">
+        <v>129</v>
+      </c>
+      <c r="D51" t="s">
+        <v>7</v>
+      </c>
+      <c r="E51" s="2">
+        <v>46135</v>
+      </c>
+      <c r="F51" s="3">
+        <v>1</v>
+      </c>
+      <c r="G51" s="3">
+        <v>0</v>
+      </c>
+      <c r="H51" s="3">
+        <v>1</v>
+      </c>
+      <c r="I51" t="s">
+        <v>4</v>
+      </c>
+      <c r="J51" t="s">
         <v>130</v>
       </c>
-      <c r="B51" t="s">
-        <v>1</v>
-      </c>
-      <c r="C51" t="s">
-        <v>26</v>
-      </c>
-      <c r="D51" t="s">
-        <v>27</v>
-      </c>
-      <c r="E51" s="2">
-        <v>46140</v>
-      </c>
-      <c r="F51" s="3">
-        <v>1</v>
-      </c>
-      <c r="G51" s="3">
-        <v>0</v>
-      </c>
-      <c r="H51" s="3">
-        <v>1</v>
-      </c>
-      <c r="I51" t="s">
-        <v>4</v>
-      </c>
-      <c r="J51" t="s">
-        <v>28</v>
-      </c>
       <c r="K51" t="s">
         <v>6</v>
       </c>
@@ -4522,7 +4513,7 @@
         <v>1</v>
       </c>
       <c r="O51" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="P51" t="s">
         <v>29</v>
@@ -4534,13 +4525,13 @@
         <v>1</v>
       </c>
       <c r="S51" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T51" t="s">
         <v>12</v>
       </c>
       <c r="U51" t="s">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="V51" t="s">
         <v>1</v>
@@ -4557,34 +4548,34 @@
     </row>
     <row r="52" spans="1:25">
       <c r="A52" t="s">
+        <v>128</v>
+      </c>
+      <c r="B52" t="s">
+        <v>1</v>
+      </c>
+      <c r="C52" t="s">
         <v>131</v>
       </c>
-      <c r="B52" t="s">
-        <v>1</v>
-      </c>
-      <c r="C52" t="s">
-        <v>132</v>
-      </c>
       <c r="D52" t="s">
-        <v>7</v>
+        <v>109</v>
       </c>
       <c r="E52" s="2">
         <v>46135</v>
       </c>
       <c r="F52" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="G52" s="3">
         <v>0</v>
       </c>
       <c r="H52" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I52" t="s">
         <v>4</v>
       </c>
       <c r="J52" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K52" t="s">
         <v>6</v>
@@ -4629,83 +4620,6 @@
         <v>1</v>
       </c>
       <c r="Y52" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="53" spans="1:25">
-      <c r="A53" t="s">
-        <v>131</v>
-      </c>
-      <c r="B53" t="s">
-        <v>1</v>
-      </c>
-      <c r="C53" t="s">
-        <v>134</v>
-      </c>
-      <c r="D53" t="s">
-        <v>112</v>
-      </c>
-      <c r="E53" s="2">
-        <v>46135</v>
-      </c>
-      <c r="F53" s="3">
-        <v>-1</v>
-      </c>
-      <c r="G53" s="3">
-        <v>0</v>
-      </c>
-      <c r="H53" s="3">
-        <v>-1</v>
-      </c>
-      <c r="I53" t="s">
-        <v>4</v>
-      </c>
-      <c r="J53" t="s">
-        <v>135</v>
-      </c>
-      <c r="K53" t="s">
-        <v>6</v>
-      </c>
-      <c r="L53" t="s">
-        <v>7</v>
-      </c>
-      <c r="M53" t="s">
-        <v>8</v>
-      </c>
-      <c r="N53" t="s">
-        <v>1</v>
-      </c>
-      <c r="O53" t="s">
-        <v>48</v>
-      </c>
-      <c r="P53" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q53" t="s">
-        <v>30</v>
-      </c>
-      <c r="R53" t="s">
-        <v>1</v>
-      </c>
-      <c r="S53" s="3">
-        <v>0</v>
-      </c>
-      <c r="T53" t="s">
-        <v>12</v>
-      </c>
-      <c r="U53" t="s">
-        <v>1</v>
-      </c>
-      <c r="V53" t="s">
-        <v>1</v>
-      </c>
-      <c r="W53" t="s">
-        <v>1</v>
-      </c>
-      <c r="X53" t="s">
-        <v>1</v>
-      </c>
-      <c r="Y53" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>